<commit_message>
pas de modif pour moi apres
</commit_message>
<xml_diff>
--- a/EXAM_FORM1_RESULTS/EXAM_FORM1_61992.xlsx
+++ b/EXAM_FORM1_RESULTS/EXAM_FORM1_61992.xlsx
@@ -516,7 +516,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>110</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -706,7 +706,7 @@
         <v>375</v>
       </c>
       <c r="K4" t="n">
-        <v>4001</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5">
@@ -733,7 +733,7 @@
         <v>14.8</v>
       </c>
       <c r="K7" t="n">
-        <v>101</v>
+        <v>10</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>

</xml_diff>